<commit_message>
Log session 2026-06-08 (T5, Woche 1) into B6_Training_Log
10 Zeilen per Voice geloggt: OAHS (L/R), Ring Dips, Lat Pulldown,
Cable Row, Lateral Raise, Reverse Fly, Y-Raises, Triceps, Biceps.
Tabelle tblLog auf A1:P12 erweitert; Category/Key per Formel.
</commit_message>
<xml_diff>
--- a/Training_2.xlsx
+++ b/Training_2.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1306" uniqueCount="735">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1352" uniqueCount="746">
   <si>
     <t>B6 — Performance-Block Dashboard (Hand Balancing / Calisthenics)</t>
   </si>
@@ -1630,6 +1630,39 @@
   </si>
   <si>
     <t>Demo-Zeile: 90 Grad schwer, je 1 saubere Rep, Handgelenk gut</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>OAHS, vor allem links, sauber</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>OAHS rechts, 3 von 5 Qualitaet</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Cable Rudern; Satz 2: 70 kg x10</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Kurzhanteln</t>
+  </si>
+  <si>
+    <t>Reverse Butterfly, Supersatz</t>
+  </si>
+  <si>
+    <t>Y-Raises, Supersatz</t>
+  </si>
+  <si>
+    <t>Kabelzug</t>
   </si>
   <si>
     <t>B6 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -2616,8 +2649,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblLog" displayName="tblLog" ref="A1:P2" totalsRowShown="0">
-  <autoFilter ref="A1:P2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblLog" displayName="tblLog" ref="A1:P12" totalsRowShown="0">
+  <autoFilter ref="A1:P12"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="DayType"/>
@@ -6664,7 +6697,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -6775,6 +6808,361 @@
         <v>533</v>
       </c>
       <c r="P2">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
+      <c r="A3" s="20">
+        <v>46181</v>
+      </c>
+      <c r="B3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>372</v>
+      </c>
+      <c r="E3">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F3" t="s">
+        <v>534</v>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+      <c r="L3">
+        <v>4</v>
+      </c>
+      <c r="O3" t="s">
+        <v>535</v>
+      </c>
+      <c r="P3">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
+      <c r="A4" s="20">
+        <v>46181</v>
+      </c>
+      <c r="B4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>372</v>
+      </c>
+      <c r="E4">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F4" t="s">
+        <v>536</v>
+      </c>
+      <c r="L4">
+        <v>3</v>
+      </c>
+      <c r="O4" t="s">
+        <v>537</v>
+      </c>
+      <c r="P4">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
+      <c r="A5" s="20">
+        <v>46181</v>
+      </c>
+      <c r="B5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>449</v>
+      </c>
+      <c r="E5">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F5" t="s">
+        <v>532</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5" t="s">
+        <v>538</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="A6" s="20">
+        <v>46181</v>
+      </c>
+      <c r="B6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>413</v>
+      </c>
+      <c r="E6">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F6" t="s">
+        <v>532</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6" t="s">
+        <v>538</v>
+      </c>
+      <c r="I6">
+        <v>65</v>
+      </c>
+      <c r="P6">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
+      <c r="A7" s="20">
+        <v>46181</v>
+      </c>
+      <c r="B7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>417</v>
+      </c>
+      <c r="E7">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F7" t="s">
+        <v>532</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7" t="s">
+        <v>538</v>
+      </c>
+      <c r="I7">
+        <v>75</v>
+      </c>
+      <c r="O7" t="s">
+        <v>539</v>
+      </c>
+      <c r="P7">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16">
+      <c r="A8" s="20">
+        <v>46181</v>
+      </c>
+      <c r="B8" t="s">
+        <v>121</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>456</v>
+      </c>
+      <c r="E8">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F8" t="s">
+        <v>532</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8" t="s">
+        <v>540</v>
+      </c>
+      <c r="I8">
+        <v>8</v>
+      </c>
+      <c r="O8" t="s">
+        <v>541</v>
+      </c>
+      <c r="P8">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16">
+      <c r="A9" s="20">
+        <v>46181</v>
+      </c>
+      <c r="B9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>424</v>
+      </c>
+      <c r="E9">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F9" t="s">
+        <v>532</v>
+      </c>
+      <c r="G9">
+        <v>3</v>
+      </c>
+      <c r="H9" t="s">
+        <v>540</v>
+      </c>
+      <c r="I9">
+        <v>25</v>
+      </c>
+      <c r="O9" t="s">
+        <v>542</v>
+      </c>
+      <c r="P9">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16">
+      <c r="A10" s="20">
+        <v>46181</v>
+      </c>
+      <c r="B10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>432</v>
+      </c>
+      <c r="E10">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F10" t="s">
+        <v>532</v>
+      </c>
+      <c r="G10">
+        <v>3</v>
+      </c>
+      <c r="H10" t="s">
+        <v>540</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="O10" t="s">
+        <v>543</v>
+      </c>
+      <c r="P10">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16">
+      <c r="A11" s="20">
+        <v>46181</v>
+      </c>
+      <c r="B11" t="s">
+        <v>121</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>460</v>
+      </c>
+      <c r="E11">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F11" t="s">
+        <v>532</v>
+      </c>
+      <c r="G11">
+        <v>3</v>
+      </c>
+      <c r="H11" t="s">
+        <v>540</v>
+      </c>
+      <c r="I11">
+        <v>16.5</v>
+      </c>
+      <c r="O11" t="s">
+        <v>544</v>
+      </c>
+      <c r="P11">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16">
+      <c r="A12" s="20">
+        <v>46181</v>
+      </c>
+      <c r="B12" t="s">
+        <v>121</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>464</v>
+      </c>
+      <c r="E12">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F12" t="s">
+        <v>532</v>
+      </c>
+      <c r="G12">
+        <v>3</v>
+      </c>
+      <c r="H12" t="s">
+        <v>538</v>
+      </c>
+      <c r="I12">
+        <v>23.5</v>
+      </c>
+      <c r="O12" t="s">
+        <v>544</v>
+      </c>
+      <c r="P12">
         <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
         <v>0</v>
       </c>
@@ -6844,7 +7232,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>534</v>
+        <v>545</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6855,20 +7243,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>535</v>
+        <v>546</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>536</v>
+        <v>547</v>
       </c>
       <c r="B4" s="11">
         <v>80.8</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>544</v>
+        <v>555</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -6877,21 +7265,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>538</v>
+        <v>549</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>545</v>
+        <v>556</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -6900,7 +7288,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -6908,7 +7296,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -6916,7 +7304,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -6925,7 +7313,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>543</v>
+        <v>554</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -6934,7 +7322,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>546</v>
+        <v>557</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -6948,27 +7336,27 @@
         <v>83</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>547</v>
+        <v>558</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>548</v>
+        <v>559</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>549</v>
+        <v>560</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>550</v>
+        <v>561</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>551</v>
+        <v>562</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>552</v>
+        <v>563</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>553</v>
+        <v>564</v>
       </c>
       <c r="B14" s="21">
         <v>250</v>
@@ -6990,7 +7378,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>554</v>
+        <v>565</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -7017,12 +7405,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>555</v>
+        <v>566</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>556</v>
+        <v>567</v>
       </c>
       <c r="B16" s="21">
         <v>200</v>
@@ -7044,12 +7432,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>557</v>
+        <v>568</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>558</v>
+        <v>569</v>
       </c>
       <c r="B17" s="21">
         <v>150</v>
@@ -7071,12 +7459,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>559</v>
+        <v>570</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>560</v>
+        <v>571</v>
       </c>
       <c r="B18" s="21">
         <v>100</v>
@@ -7098,7 +7486,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>561</v>
+        <v>572</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -7125,12 +7513,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>562</v>
+        <v>573</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>563</v>
+        <v>574</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -7141,7 +7529,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>564</v>
+        <v>575</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -7152,7 +7540,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>565</v>
+        <v>576</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -7163,7 +7551,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>566</v>
+        <v>577</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -7174,7 +7562,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>567</v>
+        <v>578</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -7219,7 +7607,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>568</v>
+        <v>579</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7228,7 +7616,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>569</v>
+        <v>580</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -7237,92 +7625,92 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>570</v>
+        <v>581</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>571</v>
+        <v>582</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>572</v>
+        <v>583</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>573</v>
+        <v>584</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>574</v>
+        <v>585</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>575</v>
+        <v>586</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>576</v>
+        <v>587</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>577</v>
+        <v>588</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>578</v>
+        <v>589</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>579</v>
+        <v>590</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>580</v>
+        <v>591</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>581</v>
+        <v>592</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>582</v>
+        <v>593</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>584</v>
+        <v>595</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>585</v>
+        <v>596</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>587</v>
+        <v>598</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>588</v>
+        <v>599</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>589</v>
+        <v>600</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>590</v>
+        <v>601</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>591</v>
+        <v>602</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>592</v>
+        <v>603</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>593</v>
+        <v>604</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>594</v>
+        <v>605</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="5" t="s">
-        <v>595</v>
+        <v>606</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -7331,7 +7719,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="4" t="s">
-        <v>596</v>
+        <v>607</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -7340,7 +7728,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="4" t="s">
-        <v>597</v>
+        <v>608</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -7349,7 +7737,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="4" t="s">
-        <v>598</v>
+        <v>609</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -7358,7 +7746,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="4" t="s">
-        <v>599</v>
+        <v>610</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -7367,7 +7755,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="4" t="s">
-        <v>600</v>
+        <v>611</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -7376,7 +7764,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="4" t="s">
-        <v>601</v>
+        <v>612</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -7385,7 +7773,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="5" t="s">
-        <v>602</v>
+        <v>613</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -7394,19 +7782,19 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="7" t="s">
-        <v>603</v>
+        <v>614</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>604</v>
+        <v>615</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>605</v>
+        <v>616</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>606</v>
+        <v>617</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>607</v>
+        <v>618</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -7414,16 +7802,16 @@
         <v>65</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>608</v>
+        <v>619</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>609</v>
+        <v>620</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>610</v>
+        <v>621</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>611</v>
+        <v>622</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -7431,16 +7819,16 @@
         <v>47</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>612</v>
+        <v>623</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>613</v>
+        <v>624</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>614</v>
+        <v>625</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>615</v>
+        <v>626</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -7448,16 +7836,16 @@
         <v>33</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>616</v>
+        <v>627</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>617</v>
+        <v>628</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>618</v>
+        <v>629</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>619</v>
+        <v>630</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -7465,21 +7853,21 @@
         <v>32</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>620</v>
+        <v>631</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>622</v>
+        <v>633</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>623</v>
+        <v>634</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="26" t="s">
-        <v>624</v>
+        <v>635</v>
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="26"/>
@@ -7488,7 +7876,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="5" t="s">
-        <v>625</v>
+        <v>636</v>
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -7497,7 +7885,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="4" t="s">
-        <v>626</v>
+        <v>637</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -7506,7 +7894,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="4" t="s">
-        <v>627</v>
+        <v>638</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -7515,7 +7903,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -7524,7 +7912,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>629</v>
+        <v>640</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -7533,7 +7921,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -7542,7 +7930,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="5" t="s">
-        <v>631</v>
+        <v>642</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -7551,104 +7939,104 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="7" t="s">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>633</v>
+        <v>644</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>634</v>
+        <v>645</v>
       </c>
       <c r="D34" s="7"/>
       <c r="E34" s="7"/>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="4" t="s">
-        <v>635</v>
+        <v>646</v>
       </c>
       <c r="B35" s="27" t="s">
-        <v>636</v>
+        <v>647</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>637</v>
+        <v>648</v>
       </c>
       <c r="D35" s="4"/>
       <c r="E35" s="4"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>638</v>
+        <v>649</v>
       </c>
       <c r="B36" s="27" t="s">
-        <v>639</v>
+        <v>650</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>640</v>
+        <v>651</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>641</v>
+        <v>652</v>
       </c>
       <c r="B37" s="27" t="s">
-        <v>642</v>
+        <v>653</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>643</v>
+        <v>654</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>644</v>
+        <v>655</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>645</v>
+        <v>656</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>646</v>
+        <v>657</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>644</v>
+        <v>655</v>
       </c>
       <c r="B39" s="27" t="s">
-        <v>647</v>
+        <v>658</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>648</v>
+        <v>659</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>649</v>
+        <v>660</v>
       </c>
       <c r="B40" s="27" t="s">
-        <v>650</v>
+        <v>661</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>651</v>
+        <v>662</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>652</v>
+        <v>663</v>
       </c>
       <c r="B41" s="27" t="s">
-        <v>653</v>
+        <v>664</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>654</v>
+        <v>665</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
@@ -7706,7 +8094,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>655</v>
+        <v>666</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7716,7 +8104,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>656</v>
+        <v>667</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -7741,12 +8129,12 @@
         <v>151</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>657</v>
+        <v>668</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>658</v>
+        <v>669</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Skill90",tblLog[Week],1)+SUMIFS(tblLog[Sets],tblLog[Category],"Planche",tblLog[Week],1)+SUMIFS(tblLog[Sets],tblLog[Category],"Push",tblLog[Week],1)</f>
@@ -7771,7 +8159,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>659</v>
+        <v>670</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Pull",tblLog[Week],1)</f>
@@ -7796,7 +8184,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>660</v>
+        <v>671</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Legs",tblLog[Week],1)</f>
@@ -7821,7 +8209,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>661</v>
+        <v>672</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTIFS(tblLog[ExerciseID],"90",tblLog[Week],1)</f>
@@ -7846,7 +8234,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>662</v>
+        <v>673</v>
       </c>
       <c r="B8" s="10">
         <f>SUMIFS(tblLog[CleanReps],tblLog[ExerciseID],"90",tblLog[Week],1)</f>
@@ -7871,7 +8259,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>663</v>
+        <v>674</v>
       </c>
       <c r="B9" s="10">
         <f>COUNTIFS(tblLog[Category],"SkillOAHS",tblLog[Week],1)</f>
@@ -7896,7 +8284,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>664</v>
+        <v>675</v>
       </c>
       <c r="B10" s="10">
         <f>COUNTIFS(tblLog[Category],"Planche",tblLog[Week],1)</f>
@@ -8021,7 +8409,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="9" t="s">
-        <v>665</v>
+        <v>676</v>
       </c>
       <c r="B15" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Core",tblLog[Week],1)</f>
@@ -8046,7 +8434,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>666</v>
+        <v>677</v>
       </c>
       <c r="B16" s="11">
         <f>IFERROR(AVERAGEIFS(tblLog[TopRPE],tblLog[Week],1),0)</f>
@@ -8071,7 +8459,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>667</v>
+        <v>678</v>
       </c>
       <c r="B17" s="11">
         <f>IFERROR(AVERAGEIFS(tblLog[Pain_0_10],tblLog[Week],1),0)</f>
@@ -8121,7 +8509,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="9" t="s">
-        <v>668</v>
+        <v>679</v>
       </c>
       <c r="B19" s="10">
         <f>COUNTIFS(tblLog[Week],1)</f>
@@ -8165,7 +8553,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>669</v>
+        <v>680</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8173,7 +8561,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>670</v>
+        <v>681</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -8181,13 +8569,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>671</v>
+        <v>682</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>672</v>
+        <v>683</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>673</v>
+        <v>684</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -8196,10 +8584,10 @@
         <v>519</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>674</v>
+        <v>685</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>675</v>
+        <v>686</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -8208,10 +8596,10 @@
         <v>520</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>676</v>
+        <v>687</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>677</v>
+        <v>688</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -8220,10 +8608,10 @@
         <v>521</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>678</v>
+        <v>689</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>679</v>
+        <v>690</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -8232,10 +8620,10 @@
         <v>358</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>680</v>
+        <v>691</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>681</v>
+        <v>692</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -8244,10 +8632,10 @@
         <v>361</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>682</v>
+        <v>693</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -8256,10 +8644,10 @@
         <v>522</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>684</v>
+        <v>695</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>685</v>
+        <v>696</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -8268,10 +8656,10 @@
         <v>523</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>686</v>
+        <v>697</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>687</v>
+        <v>698</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -8280,10 +8668,10 @@
         <v>524</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>688</v>
+        <v>699</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>689</v>
+        <v>700</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -8292,10 +8680,10 @@
         <v>525</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>686</v>
+        <v>697</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>690</v>
+        <v>701</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -8304,10 +8692,10 @@
         <v>526</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>691</v>
+        <v>702</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>692</v>
+        <v>703</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -8316,10 +8704,10 @@
         <v>527</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>693</v>
+        <v>704</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>694</v>
+        <v>705</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -8328,10 +8716,10 @@
         <v>528</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>695</v>
+        <v>706</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>696</v>
+        <v>707</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -8340,10 +8728,10 @@
         <v>529</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>686</v>
+        <v>697</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>697</v>
+        <v>708</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -8352,10 +8740,10 @@
         <v>530</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>686</v>
+        <v>697</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -8364,10 +8752,10 @@
         <v>90</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>688</v>
+        <v>699</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>699</v>
+        <v>710</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -8376,16 +8764,16 @@
         <v>531</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>700</v>
+        <v>711</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>701</v>
+        <v>712</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="5" t="s">
-        <v>702</v>
+        <v>713</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -8393,7 +8781,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>703</v>
+        <v>714</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -8401,7 +8789,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>704</v>
+        <v>715</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -8409,7 +8797,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>705</v>
+        <v>716</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -8417,7 +8805,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>706</v>
+        <v>717</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -8425,7 +8813,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>707</v>
+        <v>718</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -8433,7 +8821,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>708</v>
+        <v>719</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -8441,7 +8829,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="5" t="s">
-        <v>709</v>
+        <v>720</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -8449,13 +8837,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="7" t="s">
-        <v>710</v>
+        <v>721</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>711</v>
+        <v>722</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>712</v>
+        <v>723</v>
       </c>
       <c r="D31" s="7"/>
     </row>
@@ -8464,10 +8852,10 @@
         <v>47</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>714</v>
+        <v>725</v>
       </c>
       <c r="D32" s="4"/>
     </row>
@@ -8476,10 +8864,10 @@
         <v>33</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>715</v>
+        <v>726</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>716</v>
+        <v>727</v>
       </c>
       <c r="D33" s="4"/>
     </row>
@@ -8488,10 +8876,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>717</v>
+        <v>728</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>718</v>
+        <v>729</v>
       </c>
       <c r="D34" s="4"/>
     </row>
@@ -8500,40 +8888,40 @@
         <v>297</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>719</v>
+        <v>730</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>720</v>
+        <v>731</v>
       </c>
       <c r="D35" s="4"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="13" t="s">
-        <v>721</v>
+        <v>732</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>722</v>
+        <v>733</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>723</v>
+        <v>734</v>
       </c>
       <c r="D36" s="4"/>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="13" t="s">
-        <v>724</v>
+        <v>735</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>725</v>
+        <v>736</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>726</v>
+        <v>737</v>
       </c>
       <c r="D37" s="4"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="5" t="s">
-        <v>727</v>
+        <v>738</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -8541,7 +8929,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="4" t="s">
-        <v>728</v>
+        <v>739</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -8549,7 +8937,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="4" t="s">
-        <v>729</v>
+        <v>740</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -8557,7 +8945,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="4" t="s">
-        <v>730</v>
+        <v>741</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -8565,7 +8953,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="4" t="s">
-        <v>731</v>
+        <v>742</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -8573,7 +8961,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>732</v>
+        <v>743</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -8581,7 +8969,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="4" t="s">
-        <v>733</v>
+        <v>744</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -8589,7 +8977,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>734</v>
+        <v>745</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>

</xml_diff>

<commit_message>
Log T1 session 2026-06-10 (Woche 1) into B6_Training_Log
OAHS Line L/R (stabil, Qual 5/4), OAHS Shapes Diamond (schwach),
90 4x1 (RPE9, 2 saubere), Tuck Planche Hold 8s, Weighted Pull-up 40/35 kg.
</commit_message>
<xml_diff>
--- a/Training_2.xlsx
+++ b/Training_2.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1352" uniqueCount="746">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1378" uniqueCount="752">
   <si>
     <t>B6 — Performance-Block Dashboard (Hand Balancing / Calisthenics)</t>
   </si>
@@ -1663,6 +1663,24 @@
   </si>
   <si>
     <t>Kabelzug</t>
+  </si>
+  <si>
+    <t>OAHS Line, sehr stabile Holds links, solide</t>
+  </si>
+  <si>
+    <t>OAHS Line rechts, stabil</t>
+  </si>
+  <si>
+    <t>Diamond Shape, eher schwach</t>
+  </si>
+  <si>
+    <t>4x1 Cluster, lange Pausen; keine Kraft Bottom Position; Rep2+3 sauber (RPE7-8), Rep1+4 (8-9) unsauber</t>
+  </si>
+  <si>
+    <t>Adv-Tuck nicht moeglich; normaler Tuck Planche 8s (schwaecher als sonst)</t>
+  </si>
+  <si>
+    <t>40 kg x3, dann 35 kg x4; RPE 8-9</t>
   </si>
   <si>
     <t>B6 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -2649,8 +2667,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblLog" displayName="tblLog" ref="A1:P12" totalsRowShown="0">
-  <autoFilter ref="A1:P12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblLog" displayName="tblLog" ref="A1:P18" totalsRowShown="0">
+  <autoFilter ref="A1:P18"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="DayType"/>
@@ -6697,7 +6715,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -7163,6 +7181,234 @@
         <v>544</v>
       </c>
       <c r="P12">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16">
+      <c r="A13" s="20">
+        <v>46183</v>
+      </c>
+      <c r="B13" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13" t="s">
+        <v>372</v>
+      </c>
+      <c r="E13">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F13" t="s">
+        <v>534</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <v>5</v>
+      </c>
+      <c r="O13" t="s">
+        <v>545</v>
+      </c>
+      <c r="P13">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16">
+      <c r="A14" s="20">
+        <v>46183</v>
+      </c>
+      <c r="B14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>372</v>
+      </c>
+      <c r="E14">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F14" t="s">
+        <v>536</v>
+      </c>
+      <c r="G14">
+        <v>2</v>
+      </c>
+      <c r="K14">
+        <v>1</v>
+      </c>
+      <c r="L14">
+        <v>4</v>
+      </c>
+      <c r="O14" t="s">
+        <v>546</v>
+      </c>
+      <c r="P14">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16">
+      <c r="A15" s="20">
+        <v>46183</v>
+      </c>
+      <c r="B15" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" t="s">
+        <v>378</v>
+      </c>
+      <c r="E15">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F15" t="s">
+        <v>532</v>
+      </c>
+      <c r="G15">
+        <v>3</v>
+      </c>
+      <c r="L15">
+        <v>2</v>
+      </c>
+      <c r="O15" t="s">
+        <v>547</v>
+      </c>
+      <c r="P15">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16">
+      <c r="A16" s="20">
+        <v>46183</v>
+      </c>
+      <c r="B16" t="s">
+        <v>92</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>366</v>
+      </c>
+      <c r="E16">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F16" t="s">
+        <v>532</v>
+      </c>
+      <c r="G16">
+        <v>4</v>
+      </c>
+      <c r="H16" t="s">
+        <v>47</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>9</v>
+      </c>
+      <c r="K16">
+        <v>1</v>
+      </c>
+      <c r="N16">
+        <v>2</v>
+      </c>
+      <c r="O16" t="s">
+        <v>548</v>
+      </c>
+      <c r="P16">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16">
+      <c r="A17" s="20">
+        <v>46183</v>
+      </c>
+      <c r="B17" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>400</v>
+      </c>
+      <c r="E17">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F17" t="s">
+        <v>532</v>
+      </c>
+      <c r="G17">
+        <v>2</v>
+      </c>
+      <c r="M17">
+        <v>8</v>
+      </c>
+      <c r="O17" t="s">
+        <v>549</v>
+      </c>
+      <c r="P17">
+        <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16">
+      <c r="A18" s="20">
+        <v>46183</v>
+      </c>
+      <c r="B18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="s">
+        <v>403</v>
+      </c>
+      <c r="E18">
+        <f>IFERROR(INDEX(B6_Exercise_Library!$D$4:$D$43,MATCH([[#This Row],ExerciseID],B6_Exercise_Library!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F18" t="s">
+        <v>532</v>
+      </c>
+      <c r="G18">
+        <v>2</v>
+      </c>
+      <c r="H18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I18">
+        <v>40</v>
+      </c>
+      <c r="J18">
+        <v>9</v>
+      </c>
+      <c r="O18" t="s">
+        <v>550</v>
+      </c>
+      <c r="P18">
         <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
         <v>0</v>
       </c>
@@ -7232,7 +7478,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7243,20 +7489,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="B4" s="11">
         <v>80.8</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -7265,21 +7511,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -7288,7 +7534,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -7296,7 +7542,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -7304,7 +7550,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -7313,7 +7559,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -7322,7 +7568,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -7336,27 +7582,27 @@
         <v>83</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="B14" s="21">
         <v>250</v>
@@ -7378,7 +7624,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -7405,12 +7651,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="B16" s="21">
         <v>200</v>
@@ -7432,12 +7678,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="B17" s="21">
         <v>150</v>
@@ -7459,12 +7705,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="B18" s="21">
         <v>100</v>
@@ -7486,7 +7732,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -7513,12 +7759,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -7529,7 +7775,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -7540,7 +7786,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -7551,7 +7797,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -7562,7 +7808,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -7607,7 +7853,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7616,7 +7862,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -7625,92 +7871,92 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="5" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -7719,7 +7965,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="4" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -7728,7 +7974,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="4" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -7737,7 +7983,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="4" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -7746,7 +7992,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="4" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -7755,7 +8001,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="4" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -7764,7 +8010,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="4" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -7773,7 +8019,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="5" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -7782,19 +8028,19 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="7" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -7802,16 +8048,16 @@
         <v>65</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -7819,16 +8065,16 @@
         <v>47</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -7836,16 +8082,16 @@
         <v>33</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -7853,21 +8099,21 @@
         <v>32</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="26" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="26"/>
@@ -7876,7 +8122,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="5" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -7885,7 +8131,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="4" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -7894,7 +8140,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="4" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -7903,7 +8149,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -7912,7 +8158,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -7921,7 +8167,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -7930,7 +8176,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="5" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -7939,104 +8185,104 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="7" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
       <c r="D34" s="7"/>
       <c r="E34" s="7"/>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="4" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="B35" s="27" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="D35" s="4"/>
       <c r="E35" s="4"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="B36" s="27" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
       <c r="B37" s="27" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="B39" s="27" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="B40" s="27" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="B41" s="27" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
@@ -8094,7 +8340,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8104,7 +8350,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -8129,12 +8375,12 @@
         <v>151</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Skill90",tblLog[Week],1)+SUMIFS(tblLog[Sets],tblLog[Category],"Planche",tblLog[Week],1)+SUMIFS(tblLog[Sets],tblLog[Category],"Push",tblLog[Week],1)</f>
@@ -8159,7 +8405,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Pull",tblLog[Week],1)</f>
@@ -8184,7 +8430,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Legs",tblLog[Week],1)</f>
@@ -8209,7 +8455,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTIFS(tblLog[ExerciseID],"90",tblLog[Week],1)</f>
@@ -8234,7 +8480,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
       <c r="B8" s="10">
         <f>SUMIFS(tblLog[CleanReps],tblLog[ExerciseID],"90",tblLog[Week],1)</f>
@@ -8259,7 +8505,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
       <c r="B9" s="10">
         <f>COUNTIFS(tblLog[Category],"SkillOAHS",tblLog[Week],1)</f>
@@ -8284,7 +8530,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="B10" s="10">
         <f>COUNTIFS(tblLog[Category],"Planche",tblLog[Week],1)</f>
@@ -8409,7 +8655,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="9" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
       <c r="B15" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Core",tblLog[Week],1)</f>
@@ -8434,7 +8680,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="B16" s="11">
         <f>IFERROR(AVERAGEIFS(tblLog[TopRPE],tblLog[Week],1),0)</f>
@@ -8459,7 +8705,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="B17" s="11">
         <f>IFERROR(AVERAGEIFS(tblLog[Pain_0_10],tblLog[Week],1),0)</f>
@@ -8509,7 +8755,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="9" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="B19" s="10">
         <f>COUNTIFS(tblLog[Week],1)</f>
@@ -8553,7 +8799,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8561,7 +8807,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -8569,13 +8815,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -8584,10 +8830,10 @@
         <v>519</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -8596,10 +8842,10 @@
         <v>520</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -8608,10 +8854,10 @@
         <v>521</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -8620,10 +8866,10 @@
         <v>358</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -8632,10 +8878,10 @@
         <v>361</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>694</v>
+        <v>700</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -8644,10 +8890,10 @@
         <v>522</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -8656,10 +8902,10 @@
         <v>523</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -8668,10 +8914,10 @@
         <v>524</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -8680,10 +8926,10 @@
         <v>525</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -8692,10 +8938,10 @@
         <v>526</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -8704,10 +8950,10 @@
         <v>527</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -8716,10 +8962,10 @@
         <v>528</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -8728,10 +8974,10 @@
         <v>529</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -8740,10 +8986,10 @@
         <v>530</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -8752,10 +8998,10 @@
         <v>90</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -8764,16 +9010,16 @@
         <v>531</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>711</v>
+        <v>717</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>712</v>
+        <v>718</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="5" t="s">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -8781,7 +9027,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -8789,7 +9035,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>715</v>
+        <v>721</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -8797,7 +9043,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>716</v>
+        <v>722</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -8805,7 +9051,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>717</v>
+        <v>723</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -8813,7 +9059,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -8821,7 +9067,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>719</v>
+        <v>725</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -8829,7 +9075,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="5" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -8837,13 +9083,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="7" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>723</v>
+        <v>729</v>
       </c>
       <c r="D31" s="7"/>
     </row>
@@ -8852,10 +9098,10 @@
         <v>47</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
       <c r="D32" s="4"/>
     </row>
@@ -8864,10 +9110,10 @@
         <v>33</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>726</v>
+        <v>732</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="D33" s="4"/>
     </row>
@@ -8876,10 +9122,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>728</v>
+        <v>734</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
       <c r="D34" s="4"/>
     </row>
@@ -8888,40 +9134,40 @@
         <v>297</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
       <c r="D35" s="4"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="13" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="D36" s="4"/>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="13" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
       <c r="D37" s="4"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="5" t="s">
-        <v>738</v>
+        <v>744</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -8929,7 +9175,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="4" t="s">
-        <v>739</v>
+        <v>745</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -8937,7 +9183,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="4" t="s">
-        <v>740</v>
+        <v>746</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -8945,7 +9191,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="4" t="s">
-        <v>741</v>
+        <v>747</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -8953,7 +9199,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="4" t="s">
-        <v>742</v>
+        <v>748</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -8961,7 +9207,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>743</v>
+        <v>749</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -8969,7 +9215,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="4" t="s">
-        <v>744</v>
+        <v>750</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -8977,7 +9223,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>745</v>
+        <v>751</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>

</xml_diff>

<commit_message>
Correct/complete T1 session: Planche & WPU 4 sets, RPE fill, BW loads, pain/quality
</commit_message>
<xml_diff>
--- a/Training_2.xlsx
+++ b/Training_2.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1378" uniqueCount="752">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1378" uniqueCount="753">
   <si>
     <t>B6 — Performance-Block Dashboard (Hand Balancing / Calisthenics)</t>
   </si>
@@ -1677,10 +1677,13 @@
     <t>4x1 Cluster, lange Pausen; keine Kraft Bottom Position; Rep2+3 sauber (RPE7-8), Rep1+4 (8-9) unsauber</t>
   </si>
   <si>
-    <t>Adv-Tuck nicht moeglich; normaler Tuck Planche 8s (schwaecher als sonst)</t>
-  </si>
-  <si>
-    <t>40 kg x3, dann 35 kg x4; RPE 8-9</t>
+    <t>1x Advanced Tuck versucht (nicht moeglich) + 3x8s Tuck Planche; schwaecher als sonst</t>
+  </si>
+  <si>
+    <t>1x3@40, 3x4@35</t>
+  </si>
+  <si>
+    <t>Satz1: 40 kg x3; Satz2-4: 35 kg x4; RPE 8-9</t>
   </si>
   <si>
     <t>B6 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -7208,6 +7211,12 @@
       <c r="G13">
         <v>2</v>
       </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>8</v>
+      </c>
       <c r="K13">
         <v>1</v>
       </c>
@@ -7245,6 +7254,12 @@
       <c r="G14">
         <v>2</v>
       </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>8</v>
+      </c>
       <c r="K14">
         <v>1</v>
       </c>
@@ -7282,6 +7297,15 @@
       <c r="G15">
         <v>3</v>
       </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>8</v>
+      </c>
+      <c r="K15">
+        <v>1</v>
+      </c>
       <c r="L15">
         <v>2</v>
       </c>
@@ -7328,6 +7352,9 @@
       <c r="K16">
         <v>1</v>
       </c>
+      <c r="L16">
+        <v>3</v>
+      </c>
       <c r="N16">
         <v>2</v>
       </c>
@@ -7360,6 +7387,18 @@
         <v>532</v>
       </c>
       <c r="G17">
+        <v>4</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>8</v>
+      </c>
+      <c r="K17">
+        <v>1</v>
+      </c>
+      <c r="L17">
         <v>2</v>
       </c>
       <c r="M17">
@@ -7394,10 +7433,10 @@
         <v>532</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H18" t="s">
-        <v>32</v>
+        <v>550</v>
       </c>
       <c r="I18">
         <v>40</v>
@@ -7405,8 +7444,11 @@
       <c r="J18">
         <v>9</v>
       </c>
+      <c r="K18">
+        <v>1</v>
+      </c>
       <c r="O18" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="P18">
         <f>[[#This Row],DayType]&amp;"_W"&amp;[[#This Row],Week]</f>
@@ -7478,7 +7520,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7489,20 +7531,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B4" s="11">
         <v>80.8</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -7511,21 +7553,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -7534,7 +7576,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -7542,7 +7584,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -7550,7 +7592,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -7559,7 +7601,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -7568,7 +7610,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -7582,27 +7624,27 @@
         <v>83</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B14" s="21">
         <v>250</v>
@@ -7624,7 +7666,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -7651,12 +7693,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B16" s="21">
         <v>200</v>
@@ -7678,12 +7720,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B17" s="21">
         <v>150</v>
@@ -7705,12 +7747,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="B18" s="21">
         <v>100</v>
@@ -7732,7 +7774,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -7759,12 +7801,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -7775,7 +7817,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -7786,7 +7828,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -7797,7 +7839,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -7808,7 +7850,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -7853,7 +7895,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7862,7 +7904,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -7871,92 +7913,92 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="5" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -7965,7 +8007,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="4" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -7974,7 +8016,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="4" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -7983,7 +8025,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="4" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -7992,7 +8034,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="4" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -8001,7 +8043,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="4" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -8010,7 +8052,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="4" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -8019,7 +8061,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="5" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -8028,19 +8070,19 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="7" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -8048,16 +8090,16 @@
         <v>65</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -8065,16 +8107,16 @@
         <v>47</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -8082,16 +8124,16 @@
         <v>33</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -8099,21 +8141,21 @@
         <v>32</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="26" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="26"/>
@@ -8122,7 +8164,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="5" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -8131,7 +8173,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="4" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -8140,7 +8182,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="4" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -8149,7 +8191,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -8158,7 +8200,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -8167,7 +8209,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -8176,7 +8218,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="5" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -8185,104 +8227,104 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="7" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D34" s="7"/>
       <c r="E34" s="7"/>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="4" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B35" s="27" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="D35" s="4"/>
       <c r="E35" s="4"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B36" s="27" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B37" s="27" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B39" s="27" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B40" s="27" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B41" s="27" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
@@ -8340,7 +8382,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8350,7 +8392,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -8375,12 +8417,12 @@
         <v>151</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Skill90",tblLog[Week],1)+SUMIFS(tblLog[Sets],tblLog[Category],"Planche",tblLog[Week],1)+SUMIFS(tblLog[Sets],tblLog[Category],"Push",tblLog[Week],1)</f>
@@ -8405,7 +8447,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Pull",tblLog[Week],1)</f>
@@ -8430,7 +8472,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Legs",tblLog[Week],1)</f>
@@ -8455,7 +8497,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTIFS(tblLog[ExerciseID],"90",tblLog[Week],1)</f>
@@ -8480,7 +8522,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B8" s="10">
         <f>SUMIFS(tblLog[CleanReps],tblLog[ExerciseID],"90",tblLog[Week],1)</f>
@@ -8505,7 +8547,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B9" s="10">
         <f>COUNTIFS(tblLog[Category],"SkillOAHS",tblLog[Week],1)</f>
@@ -8530,7 +8572,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="B10" s="10">
         <f>COUNTIFS(tblLog[Category],"Planche",tblLog[Week],1)</f>
@@ -8655,7 +8697,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="9" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="B15" s="11">
         <f>SUMIFS(tblLog[Sets],tblLog[Category],"Core",tblLog[Week],1)</f>
@@ -8680,7 +8722,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B16" s="11">
         <f>IFERROR(AVERAGEIFS(tblLog[TopRPE],tblLog[Week],1),0)</f>
@@ -8705,7 +8747,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="B17" s="11">
         <f>IFERROR(AVERAGEIFS(tblLog[Pain_0_10],tblLog[Week],1),0)</f>
@@ -8755,7 +8797,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="9" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B19" s="10">
         <f>COUNTIFS(tblLog[Week],1)</f>
@@ -8799,7 +8841,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8807,7 +8849,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -8815,13 +8857,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -8830,10 +8872,10 @@
         <v>519</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -8842,10 +8884,10 @@
         <v>520</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -8854,10 +8896,10 @@
         <v>521</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -8866,10 +8908,10 @@
         <v>358</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -8878,10 +8920,10 @@
         <v>361</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -8890,10 +8932,10 @@
         <v>522</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -8902,10 +8944,10 @@
         <v>523</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -8914,10 +8956,10 @@
         <v>524</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -8926,10 +8968,10 @@
         <v>525</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -8938,10 +8980,10 @@
         <v>526</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -8950,10 +8992,10 @@
         <v>527</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -8962,10 +9004,10 @@
         <v>528</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -8974,10 +9016,10 @@
         <v>529</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -8986,10 +9028,10 @@
         <v>530</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -8998,10 +9040,10 @@
         <v>90</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -9010,16 +9052,16 @@
         <v>531</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="5" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -9027,7 +9069,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -9035,7 +9077,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -9043,7 +9085,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -9051,7 +9093,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -9059,7 +9101,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -9067,7 +9109,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -9075,7 +9117,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="5" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -9083,13 +9125,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="7" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="D31" s="7"/>
     </row>
@@ -9098,10 +9140,10 @@
         <v>47</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="D32" s="4"/>
     </row>
@@ -9110,10 +9152,10 @@
         <v>33</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="D33" s="4"/>
     </row>
@@ -9122,10 +9164,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="D34" s="4"/>
     </row>
@@ -9134,40 +9176,40 @@
         <v>297</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="D35" s="4"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="13" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="D36" s="4"/>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="13" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="D37" s="4"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="5" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -9175,7 +9217,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="4" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -9183,7 +9225,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="4" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -9191,7 +9233,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="4" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -9199,7 +9241,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="4" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -9207,7 +9249,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -9215,7 +9257,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="4" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -9223,7 +9265,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>

</xml_diff>